<commit_message>
We now have more tops in place, for delve, exploration, so on and so forth.
</commit_message>
<xml_diff>
--- a/resources/data-imports/Quests/guide-quests.xlsx
+++ b/resources/data-imports/Quests/guide-quests.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="393">
   <si>
     <t>id</t>
   </si>
@@ -188,6 +188,42 @@
     <t>required_delve_pack_size</t>
   </si>
   <si>
+    <t>required_batch_crafting_type</t>
+  </si>
+  <si>
+    <t>required_batch_crafting_hours</t>
+  </si>
+  <si>
+    <t>required_item_1_source</t>
+  </si>
+  <si>
+    <t>required_item_1_name</t>
+  </si>
+  <si>
+    <t>required_item_1_type</t>
+  </si>
+  <si>
+    <t>required_item_1_amount</t>
+  </si>
+  <si>
+    <t>required_item_1_must_be_enchanted</t>
+  </si>
+  <si>
+    <t>required_item_2_source</t>
+  </si>
+  <si>
+    <t>required_item_2_name</t>
+  </si>
+  <si>
+    <t>required_item_2_type</t>
+  </si>
+  <si>
+    <t>required_item_2_amount</t>
+  </si>
+  <si>
+    <t>required_item_2_must_be_enchanted</t>
+  </si>
+  <si>
     <t>Welcome to Tlessa</t>
   </si>
   <si>
@@ -1035,6 +1071,129 @@
   </si>
   <si>
     <t>&lt;p&gt;Complete the remaining quests until you reach the end of The Emerald Mirror story line: The beating heart at the center.&lt;/p&gt;&lt;p&gt;Survive a pack size of 10 or greater for 2 or more hours in Delve.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Automating the smithing process</t>
+  </si>
+  <si>
+    <t>You are exhausted, depleted, and emotionally drained from helping the local blacksmith. This is what he does all day, every day. You think to yourself as you sit in the inn: there has to be a better way to do this. You devise a plan to introduce the blacksmith to a form of automation …</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Welcome to Batch Crafting. In this tutorial, we are going to help that blacksmith by batch crafting items for experience. We are going to do this for an hour.&lt;/p&gt;&lt;p&gt;Batch crafting is a system you can learn more about in the help docs. It allows players to automate the levelling experience of crafting, as well as batch craft specific items.&lt;/p&gt;&lt;p&gt;Batch crafted items go to a few different places:&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Alchemy items go to your alchemy bag.&lt;/li&gt;&lt;li&gt;Weapons and armour go to a special set called Crafted Items in your inventory. This can hold a maximum of 2,000 items. You may only remove items from here.&lt;/li&gt;&lt;li&gt;Trinkets go in your inventory.&lt;/li&gt;&lt;li&gt;Items you apply holy oils to go into your inventory.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;We will cover this more in the next guide quest. For now, let’s craft and explore.&lt;/p&gt;&lt;p&gt;Crafting and enchanting are such integral aspects of the gear treadmill in Tlessa that you cannot survive on shop gear or found gear for very long. So we are going to speed up our crafting and introduce Batch Crafting.&lt;/p&gt;&lt;p&gt;Keep all the items you craft.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;From the Craft and Enchant drop-down, select Batch Craft. Then leave everything as it is, and select: Keep Highest Level Crafted At The End for disposition.&lt;/p&gt;&lt;p&gt;Click Batch Craft. Might as well also set up some exploration while you’re here, no?&lt;/p&gt;&lt;p&gt;This is going to craft items until one of five things happens:&lt;/p&gt;&lt;ol&gt;&lt;li&gt;You run out of gold.&lt;/li&gt;&lt;li&gt;You run out of crafted inventory space (more on that in the next guide quest).&lt;/li&gt;&lt;li&gt;You die for some reason.&lt;/li&gt;&lt;li&gt;You max out the crafting skill or skills.&lt;/li&gt;&lt;li&gt;You decide to stop it.&lt;/li&gt;&lt;/ol&gt;&lt;p&gt;For now, just craft for an hour. You’ll know when to stop it because the guide quest will be ready to hand in.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;From the main option drop-down, select Craft, then Batch Craft. Then leave everything as it is, and select: Keep Highest Level Crafted At The End for disposition.&lt;/p&gt;&lt;p&gt;Click Batch Craft. Might as well also set up some exploration while you’re here, no?&lt;/p&gt;&lt;p&gt;This is going to craft items until one of five things happens:&lt;/p&gt;&lt;ol&gt;&lt;li&gt;You run out of gold.&lt;/li&gt;&lt;li&gt;You run out of crafted inventory space (more on that in the next guide quest).&lt;/li&gt;&lt;li&gt;You die for some reason.&lt;/li&gt;&lt;li&gt;You max out the crafting skill or skills.&lt;/li&gt;&lt;li&gt;You decide to stop it.&lt;/li&gt;&lt;/ol&gt;&lt;p&gt;For now, just craft for an hour. You’ll know when to stop it because the guide quest will be ready to hand in.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>craft</t>
+  </si>
+  <si>
+    <t>Effeciency is key</t>
+  </si>
+  <si>
+    <t>The Enchantress and the Blacksmith are quite impressed. As they talk among themselves about the grand plans they have for their individual enterprises, a man appears to move through the shadows. You chase him down to the back alley and see him: young, handsome, and unmistakably the Guide.&lt;br /&gt; &lt;br /&gt; “Why haven’t you been busy?” he scoffs.&lt;br /&gt; &lt;br /&gt; You ask him what he wants, and he states, “I need some weapons and some enchanted armour for a fight I’m going into, a fight to get us some answers. I fear the worst might be true.”&lt;br /&gt; &lt;br /&gt; You have a look of concern on your face but agree anyway, hoping he might tell you something.</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;We have used batch crafting, and we have used batch craft and enchant. Now let’s use the system to create very specific items. First, you will use Craft and batch craft X items. Then you will turn around and do the same thing for Craft and Enchant, but select the item. It does not matter which enchantments you select; the item just has to have two enchants. Once that’s done and the items are in your inventory, the quest will be done.&lt;/p&gt;&lt;p&gt;That’s how we batch craft items, enchant them, and create specific quantities.&lt;/p&gt;&lt;p&gt;I’ll be back again, child, when we do alchemy and dive into holy oils. For now, continue on your journeys.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Just as before, let’s open Batch Craft. This time, select Craft, and then at the bottom, where it says Craft Mode, choose Specific Type and enter the details for the items that do not need enchantments. Let that craft, then do the same thing for Craft and Enchant and fill in the details for the enchanted item.&lt;/p&gt;&lt;p&gt;The enchantments you choose are yours to choose. Just make sure you choose both a prefix and a suffix.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>craft_and_enchant</t>
+  </si>
+  <si>
+    <t>inventory</t>
+  </si>
+  <si>
+    <t>Paladin's Oath Chest</t>
+  </si>
+  <si>
+    <t>Body</t>
+  </si>
+  <si>
+    <t>Diamond Mace</t>
+  </si>
+  <si>
+    <t>Mace</t>
+  </si>
+  <si>
+    <t>A request from The Guide</t>
+  </si>
+  <si>
+    <t>“Mixing potions, are we?” You look up from your studies and see the Guide. What could he want this time? Perhaps answers as to where he went with the weapons and armour you gave him last time?&lt;br /&gt; &lt;br /&gt; You start to ask, but he interrupts you.&lt;br /&gt; &lt;br /&gt; “I need you to figure out how to speed this up. I need items created for this battle.”&lt;br /&gt; &lt;br /&gt; You ask him if he even went to the battle.&lt;br /&gt; &lt;br /&gt; “No, I have been waiting for you to craft something for me. Then I am off!”&lt;br /&gt; &lt;br /&gt; You look confused.</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Remember Batch Crafting? Yeah, we’re going to do that again, but this time for alchemy items. The same principle applies: you can select Keep, Keep the Best, or whatever else. We just need you to do this for an hour.&lt;/p&gt;&lt;p&gt;Batch crafting alchemy items works the same way as crafting or enchanting, but these items go into your Alchemy Bag, which has its own inventory limit of 150 items. You will continue to craft six per minute until you reach the full amount if you choose to keep them. I would sell or keep the highest-level one after that. Up to you.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;By now, we know how to get to Batch Crafting, so let’s select Alchemy from the Crafting Type and choose either Keep Highest Level Crafted At The End or Sell.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>alchemy</t>
+  </si>
+  <si>
+    <t>The alure of The Entranchtress</t>
+  </si>
+  <si>
+    <t>The Enchantress watches you as you manage to craft an item and then manually enchant it. She watches you do this for a while. Maybe you could automate the crafting aspect a bit, like you showed the Blacksmith. It has made his life a lot easier; he can charge top-tier coin for mass-produced, top-tier weapons and armour.&lt;br /&gt; &lt;br /&gt; “Child,” she asks as you stop and look over, “is there not an easier way to do this task?”&lt;br /&gt; &lt;br /&gt; You think for a moment and then smile.</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;So there are two parts to this. First, we have to go to your inventory and see what it created for you. Since you told it to keep only the best, remove those items from your inventory set called Crafted Items. See the instructions for how to do this. These items should end up in your inventory, assuming you have the space, that is.&lt;/p&gt;&lt;p&gt;Next, we’ll combine crafting and enchanting for the next aspect.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Just as before, open Batch Craft. Instead of Craft, in the top select, choose Craft and Enchant and do it for experience. Choose to keep the highest-level crafted item at the end.&lt;/p&gt;&lt;p&gt;Click Batch Craft. Might as well also set up some exploration while you’re here, no?&lt;/p&gt;&lt;p&gt;This is going to craft and then enchant six sets until one of five things happens:&lt;/p&gt;&lt;ol&gt;&lt;li&gt;You run out of gold.&lt;/li&gt;&lt;li&gt;You run out of crafted inventory space (more on that in the next guide quest).&lt;/li&gt;&lt;li&gt;You die for some reason.&lt;/li&gt;&lt;li&gt;You max out the crafting skill or skills.&lt;/li&gt;&lt;li&gt;You decide to stop it.&lt;/li&gt;&lt;/ol&gt;&lt;p&gt;For now, just craft and enchant for an hour. You’ll know when to stop it because the guide quest will be ready to hand in.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>More errands for The Guide</t>
+  </si>
+  <si>
+    <t>You whiz through the alchemy items and craft many, basically automating the entire process and making it so much easier. It has been almost two weeks with no sign of the Guide. Just as you’re about to head out for an adventure and wait for him, he appears.&lt;br /&gt; &lt;br /&gt; “Hello, child,” he greets you warmly.&lt;br /&gt; &lt;br /&gt; You step aside and let him in, then ask him what this fight is all about.&lt;br /&gt; &lt;br /&gt; “There is something happening, child. A gate has been found, and until I know more, I have to keep you busy. I need some alchemy items, and I have a list here. Let’s get these created, shall we?”&lt;br /&gt; &lt;br /&gt; You stare at his list and then at him. What are you? His whipping boy?</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Now we know how to craft, craft and enchant, create multiple items, and craft alchemy items. Now we’re going to create very specific alchemy items for the Guide.&lt;/p&gt;&lt;p&gt;Look at what he wants. When you set up alchemy, choose Keep and Craft Amount to craft a specific amount.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;When setting up alchemy for batch crafting, select Keep, select Specific Amount, and create what the Guide wants.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>alchemy_bag</t>
+  </si>
+  <si>
+    <t>Mixtures and Concoctions</t>
+  </si>
+  <si>
+    <t>Increases Alchemy Skill</t>
+  </si>
+  <si>
+    <t>The Gates Are Opening</t>
+  </si>
+  <si>
+    <t>You’re sitting alone in a room in an abandoned house, trying to recover from the last adventure you were on and mending your wounds, when an older man’s voice appears out of nowhere and a man walks from the shadows.&lt;br /&gt; &lt;br /&gt; “Have you seen where I put my oils? My gear isn’t holding up in this fight.”&lt;br /&gt; &lt;br /&gt; You look more closely and realize it is the Guide, but older and more frail-looking. You ask him what happened.&lt;br /&gt; &lt;br /&gt; “The gates, child. They are opening. He will walk again, and chaos will come.”&lt;br /&gt; &lt;br /&gt; You look at him with shock on your face.&lt;br /&gt; &lt;br /&gt; “Alas, you are not prepared yet to handle what comes once those gates are opened. However, you can be. You’ll need some oil and some gear.”</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;By now, you have applied some holy oils to your equipment, but did you know you can do this in batch? Yes, you can use Batch Craft to do this by selecting Holy Oils.&lt;/p&gt;&lt;p&gt;This will take the oils and apply them to selected gear until all the holy stacks on the items are filled, or until you run out of currencies or oils.&lt;/p&gt;&lt;p&gt;So you’ll need to craft some oils. Might as well batch craft that, and then use the Holy Oils section to apply the oils to your selected items. As long as you have the required holy stacks, you are good no matter how you do this.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ul&gt;&lt;li&gt;Use batch crafting if needed to craft some items.&lt;/li&gt;&lt;li&gt;Use Craft Amount on alchemy items to craft some oils.&lt;/li&gt;&lt;li&gt;Use Holy Oils from Batch Crafting to select the items and the oils, then start the process.&lt;/li&gt;&lt;/ul&gt;</t>
+  </si>
+  <si>
+    <t>Where do we go from here?</t>
+  </si>
+  <si>
+    <t>You stand before an old altar in ruins in the middle of nowhere. The shadows of your mind dance around, and you see it clearly before you: a vision.&lt;br /&gt; &lt;br /&gt; Before you stands the Guide, bloodied and broken. His voice reaches out across time and space, echoing in your ear: “Child, the gates are opening. The prince will walk. I need you to hurry up with those damn trinkets …”</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;The last aspect of Batch Crafting is Trinketry. These will appear in your Crafted Items set, and we will craft six at a time for experience. You can’t craft multiples of these because it doesn’t make sense, so you might as well keep the best one.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>&lt;ul&gt;&lt;li&gt;Use batch crafting to craft trinkets for experience. Keep the best one, and do this for an hour.&lt;/li&gt;&lt;/ul&gt;</t>
+  </si>
+  <si>
+    <t>trinketry</t>
   </si>
 </sst>
 </file>
@@ -1374,7 +1533,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:BH51"/>
+  <dimension ref="A1:BT58"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="3.428" bestFit="true" customWidth="true" style="0"/>
@@ -1437,9 +1596,21 @@
     <col min="58" max="58" width="23.423" bestFit="true" customWidth="true" style="0"/>
     <col min="59" max="59" width="34.135" bestFit="true" customWidth="true" style="0"/>
     <col min="60" max="60" width="29.421" bestFit="true" customWidth="true" style="0"/>
+    <col min="61" max="61" width="34.135" bestFit="true" customWidth="true" style="0"/>
+    <col min="62" max="62" width="35.277" bestFit="true" customWidth="true" style="0"/>
+    <col min="63" max="63" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="64" max="64" width="29.421" bestFit="true" customWidth="true" style="0"/>
+    <col min="65" max="65" width="28.136" bestFit="true" customWidth="true" style="0"/>
+    <col min="66" max="66" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="67" max="67" width="39.99" bestFit="true" customWidth="true" style="0"/>
+    <col min="68" max="68" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="69" max="69" width="24.708" bestFit="true" customWidth="true" style="0"/>
+    <col min="70" max="70" width="24.708" bestFit="true" customWidth="true" style="0"/>
+    <col min="71" max="71" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="72" max="72" width="39.99" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:60">
+    <row r="1" spans="1:72">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1611,25 +1782,61 @@
       <c r="BH1" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="2" spans="1:60">
+      <c r="BI1" t="s">
+        <v>57</v>
+      </c>
+      <c r="BJ1" t="s">
+        <v>58</v>
+      </c>
+      <c r="BK1" t="s">
+        <v>59</v>
+      </c>
+      <c r="BL1" t="s">
+        <v>60</v>
+      </c>
+      <c r="BM1" t="s">
+        <v>61</v>
+      </c>
+      <c r="BN1" t="s">
+        <v>62</v>
+      </c>
+      <c r="BO1" t="s">
+        <v>63</v>
+      </c>
+      <c r="BP1" t="s">
+        <v>64</v>
+      </c>
+      <c r="BQ1" t="s">
+        <v>65</v>
+      </c>
+      <c r="BR1" t="s">
+        <v>66</v>
+      </c>
+      <c r="BS1" t="s">
+        <v>67</v>
+      </c>
+      <c r="BT1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:72">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="D2" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="E2" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="F2" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="G2">
         <v>2</v>
@@ -1641,30 +1848,30 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:60">
+    <row r="3" spans="1:72">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="C3" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="D3" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="E3" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="F3" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="G3">
         <v>10</v>
       </c>
       <c r="Q3" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="R3">
         <v>1</v>
@@ -1676,36 +1883,36 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:60">
+    <row r="4" spans="1:72">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="C4" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="D4" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="E4" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="F4" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="G4">
         <v>30</v>
       </c>
       <c r="I4" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="J4">
         <v>10</v>
       </c>
       <c r="K4" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="L4">
         <v>15</v>
@@ -1720,45 +1927,45 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:60">
+    <row r="5" spans="1:72">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="D5" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="E5" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="F5" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="G5">
         <v>50</v>
       </c>
       <c r="I5" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="J5">
         <v>5</v>
       </c>
       <c r="K5" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="U5" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="V5" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="AS5">
         <v>1000</v>
@@ -1767,42 +1974,42 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:60">
+    <row r="6" spans="1:72">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="C6" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="D6" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="E6" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="F6" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="G6">
         <v>60</v>
       </c>
       <c r="I6" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="J6">
         <v>5</v>
       </c>
       <c r="K6" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="L6">
         <v>15</v>
       </c>
       <c r="U6" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="AM6">
         <v>125</v>
@@ -1814,36 +2021,36 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:60">
+    <row r="7" spans="1:72">
       <c r="A7">
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="C7" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="D7" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="E7" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="F7" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="G7">
         <v>120</v>
       </c>
       <c r="I7" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="J7">
         <v>15</v>
       </c>
       <c r="K7" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="L7">
         <v>5</v>
@@ -1855,7 +2062,7 @@
         <v>10</v>
       </c>
       <c r="U7" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="X7">
         <v>500</v>
@@ -1876,33 +2083,33 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:60">
+    <row r="8" spans="1:72">
       <c r="A8">
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="C8" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="D8" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="E8" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="F8" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="Q8" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="R8">
         <v>3</v>
       </c>
       <c r="T8" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="AQ8">
         <v>1000</v>
@@ -1917,33 +2124,33 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:60">
+    <row r="9" spans="1:72">
       <c r="A9">
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="C9" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="D9" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="E9" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="F9" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="I9" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="J9">
         <v>50</v>
       </c>
       <c r="T9" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="AQ9">
         <v>2500</v>
@@ -1958,39 +2165,39 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:60">
+    <row r="10" spans="1:72">
       <c r="A10">
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="C10" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="D10" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="E10" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="F10" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="G10">
         <v>300</v>
       </c>
       <c r="Q10" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="R10">
         <v>2</v>
       </c>
       <c r="S10" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="U10" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="AQ10">
         <v>1000</v>
@@ -2002,24 +2209,24 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:60">
+    <row r="11" spans="1:72">
       <c r="A11">
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="C11" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="D11" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="E11" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="F11" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="O11">
         <v>1</v>
@@ -2034,24 +2241,24 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="1:60">
+    <row r="12" spans="1:72">
       <c r="A12">
         <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="C12" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="D12" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="E12" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="F12" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="AB12">
         <v>1</v>
@@ -2069,33 +2276,33 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:60">
+    <row r="13" spans="1:72">
       <c r="A13">
         <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="C13" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="D13" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="E13" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="F13" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="I13" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="J13">
         <v>25</v>
       </c>
       <c r="K13" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="L13">
         <v>5</v>
@@ -2107,7 +2314,7 @@
         <v>500</v>
       </c>
       <c r="AG13" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="AH13">
         <v>1</v>
@@ -2119,24 +2326,24 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:60">
+    <row r="14" spans="1:72">
       <c r="A14">
         <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="C14" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="D14" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="E14" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="F14" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="AC14">
         <v>75</v>
@@ -2145,7 +2352,7 @@
         <v>2000</v>
       </c>
       <c r="AG14" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="AH14">
         <v>2</v>
@@ -2157,33 +2364,33 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:60">
+    <row r="15" spans="1:72">
       <c r="A15">
         <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="C15" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="D15" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="E15" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F15" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="I15" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="J15">
         <v>25</v>
       </c>
       <c r="K15" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="L15">
         <v>50</v>
@@ -2195,7 +2402,7 @@
         <v>10</v>
       </c>
       <c r="T15" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="AC15">
         <v>100</v>
@@ -2204,7 +2411,7 @@
         <v>3000</v>
       </c>
       <c r="AG15" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="AH15">
         <v>1</v>
@@ -2216,36 +2423,36 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="1:60">
+    <row r="16" spans="1:72">
       <c r="A16">
         <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="C16" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D16" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="E16" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="F16" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="G16">
         <v>500</v>
       </c>
       <c r="I16" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="J16">
         <v>100</v>
       </c>
       <c r="K16" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="L16">
         <v>50</v>
@@ -2257,22 +2464,22 @@
         <v>100</v>
       </c>
       <c r="Q16" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="R16">
         <v>3</v>
       </c>
       <c r="S16" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="T16" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="U16" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="V16" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="X16">
         <v>25000</v>
@@ -2287,30 +2494,30 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" spans="1:60">
+    <row r="17" spans="1:72">
       <c r="A17">
         <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="C17" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="D17" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="E17" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="F17" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="G17">
         <v>600</v>
       </c>
       <c r="I17" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="J17">
         <v>3</v>
@@ -2334,30 +2541,30 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:60">
+    <row r="18" spans="1:72">
       <c r="A18">
         <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="C18" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="D18" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="E18" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="F18" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="G18">
         <v>1000</v>
       </c>
       <c r="K18" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="L18">
         <v>400</v>
@@ -2375,7 +2582,7 @@
         <v>30</v>
       </c>
       <c r="T18" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="AI18">
         <v>6000</v>
@@ -2393,39 +2600,39 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="19" spans="1:60">
+    <row r="19" spans="1:72">
       <c r="A19">
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="C19" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="D19" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="E19" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="F19" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="G19">
         <v>1500</v>
       </c>
       <c r="Q19" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="R19">
         <v>2</v>
       </c>
       <c r="S19" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="U19" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="AI19">
         <v>7000</v>
@@ -2437,30 +2644,30 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="20" spans="1:60">
+    <row r="20" spans="1:72">
       <c r="A20">
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="C20" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="D20" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="E20" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="F20" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="G20">
         <v>2000</v>
       </c>
       <c r="T20" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="AS20">
         <v>2000000000</v>
@@ -2469,30 +2676,30 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="21" spans="1:60">
+    <row r="21" spans="1:72">
       <c r="A21">
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="C21" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="D21" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="E21" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="F21" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="G21">
         <v>2500</v>
       </c>
       <c r="I21" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="J21">
         <v>50</v>
@@ -2504,7 +2711,7 @@
         <v>50</v>
       </c>
       <c r="Q21" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="R21">
         <v>5</v>
@@ -2519,7 +2726,7 @@
         <v>20000</v>
       </c>
       <c r="AE21" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="AF21">
         <v>5</v>
@@ -2537,24 +2744,24 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="22" spans="1:60">
+    <row r="22" spans="1:72">
       <c r="A22">
         <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="C22" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="D22" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="E22" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="F22" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="AS22">
         <v>100000</v>
@@ -2569,27 +2776,27 @@
         <v>3</v>
       </c>
       <c r="BA22" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="23" spans="1:60">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="23" spans="1:72">
       <c r="A23">
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="C23" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="D23" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="E23" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="F23" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="AS23">
         <v>100000</v>
@@ -2598,7 +2805,7 @@
         <v>75</v>
       </c>
       <c r="AU23" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="AW23">
         <v>25</v>
@@ -2610,27 +2817,27 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="24" spans="1:60">
+    <row r="24" spans="1:72">
       <c r="A24">
         <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="C24" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="D24" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="E24" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="F24" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="T24" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="AQ24">
         <v>5000</v>
@@ -2645,7 +2852,7 @@
         <v>100</v>
       </c>
       <c r="AU24" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="AW24">
         <v>25</v>
@@ -2654,27 +2861,27 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:60">
+    <row r="25" spans="1:72">
       <c r="A25">
         <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="C25" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="D25" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="E25" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="F25" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="T25" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="AQ25">
         <v>1000</v>
@@ -2689,7 +2896,7 @@
         <v>100</v>
       </c>
       <c r="AU25" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="AW25">
         <v>25</v>
@@ -2698,27 +2905,27 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:60">
+    <row r="26" spans="1:72">
       <c r="A26">
         <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="C26" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="D26" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="E26" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="F26" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="T26" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="AQ26">
         <v>2000</v>
@@ -2733,7 +2940,7 @@
         <v>100</v>
       </c>
       <c r="AU26" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="AW26">
         <v>25</v>
@@ -2742,27 +2949,27 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:60">
+    <row r="27" spans="1:72">
       <c r="A27">
         <v>32</v>
       </c>
       <c r="B27" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="C27" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="D27" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="E27" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="F27" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="T27" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="AB27">
         <v>1</v>
@@ -2774,7 +2981,7 @@
         <v>500</v>
       </c>
       <c r="AG27" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="AH27">
         <v>1</v>
@@ -2792,7 +2999,7 @@
         <v>100</v>
       </c>
       <c r="AU27" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="AW27">
         <v>25</v>
@@ -2801,33 +3008,33 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:60">
+    <row r="28" spans="1:72">
       <c r="A28">
         <v>33</v>
       </c>
       <c r="B28" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="C28" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="D28" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="E28" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="F28" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="S28" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="T28" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="U28" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="AQ28">
         <v>25000</v>
@@ -2842,30 +3049,30 @@
         <v>2000</v>
       </c>
       <c r="BA28" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="29" spans="1:60">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="29" spans="1:72">
       <c r="A29">
         <v>34</v>
       </c>
       <c r="B29" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="C29" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="D29" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="E29" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="F29" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="Q29" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="R29">
         <v>2</v>
@@ -2883,30 +3090,30 @@
         <v>2000</v>
       </c>
       <c r="BE29" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="30" spans="1:60">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="30" spans="1:72">
       <c r="A30">
         <v>35</v>
       </c>
       <c r="B30" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="C30" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="D30" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="E30" t="s">
+        <v>239</v>
+      </c>
+      <c r="F30" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q30" t="s">
         <v>227</v>
-      </c>
-      <c r="F30" t="s">
-        <v>228</v>
-      </c>
-      <c r="Q30" t="s">
-        <v>215</v>
       </c>
       <c r="R30">
         <v>5</v>
@@ -2924,30 +3131,30 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="31" spans="1:60">
+    <row r="31" spans="1:72">
       <c r="A31">
         <v>36</v>
       </c>
       <c r="B31" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
       <c r="C31" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="D31" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="E31" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="F31" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="S31" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="T31" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="AQ31">
         <v>25000</v>
@@ -2962,30 +3169,30 @@
         <v>2000</v>
       </c>
       <c r="BA31" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="32" spans="1:60">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="32" spans="1:72">
       <c r="A32">
         <v>37</v>
       </c>
       <c r="B32" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="C32" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="D32" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="E32" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="F32" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="I32" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="J32">
         <v>200</v>
@@ -3003,27 +3210,27 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="33" spans="1:60">
+    <row r="33" spans="1:72">
       <c r="A33">
         <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="C33" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="D33" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="E33" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="F33" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="T33" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="Z33">
         <v>5000</v>
@@ -3044,24 +3251,24 @@
         <v>40</v>
       </c>
     </row>
-    <row r="34" spans="1:60">
+    <row r="34" spans="1:72">
       <c r="A34">
         <v>39</v>
       </c>
       <c r="B34" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="C34" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="D34" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="E34" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="F34" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="AQ34">
         <v>50000</v>
@@ -3076,30 +3283,30 @@
         <v>5000</v>
       </c>
       <c r="BE34" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="35" spans="1:60">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="35" spans="1:72">
       <c r="A35">
         <v>40</v>
       </c>
       <c r="B35" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="C35" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="D35" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="E35" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
       <c r="F35" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="I35" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="J35">
         <v>25</v>
@@ -3117,27 +3324,27 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="36" spans="1:60">
+    <row r="36" spans="1:72">
       <c r="A36">
         <v>41</v>
       </c>
       <c r="B36" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="C36" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="D36" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="E36" t="s">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="F36" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="Q36" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="R36">
         <v>5</v>
@@ -3161,33 +3368,33 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:60">
+    <row r="37" spans="1:72">
       <c r="A37">
         <v>42</v>
       </c>
       <c r="B37" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="C37" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
       <c r="D37" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="E37" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="F37" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="I37" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="J37">
         <v>75</v>
       </c>
       <c r="T37" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
       <c r="AQ37">
         <v>150000</v>
@@ -3202,27 +3409,27 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="38" spans="1:60">
+    <row r="38" spans="1:72">
       <c r="A38">
         <v>43</v>
       </c>
       <c r="B38" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="C38" t="s">
+        <v>279</v>
+      </c>
+      <c r="D38" t="s">
+        <v>280</v>
+      </c>
+      <c r="E38" t="s">
+        <v>281</v>
+      </c>
+      <c r="F38" t="s">
+        <v>282</v>
+      </c>
+      <c r="I38" t="s">
         <v>267</v>
-      </c>
-      <c r="D38" t="s">
-        <v>268</v>
-      </c>
-      <c r="E38" t="s">
-        <v>269</v>
-      </c>
-      <c r="F38" t="s">
-        <v>270</v>
-      </c>
-      <c r="I38" t="s">
-        <v>255</v>
       </c>
       <c r="J38">
         <v>150</v>
@@ -3243,13 +3450,13 @@
         <v>50000</v>
       </c>
       <c r="AE38" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
       <c r="AF38">
         <v>30</v>
       </c>
       <c r="AG38" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="AH38">
         <v>4</v>
@@ -3267,27 +3474,27 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="39" spans="1:60">
+    <row r="39" spans="1:72">
       <c r="A39">
         <v>44</v>
       </c>
       <c r="B39" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="C39" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="D39" t="s">
-        <v>275</v>
+        <v>287</v>
       </c>
       <c r="E39" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="F39" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="I39" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="J39">
         <v>300</v>
@@ -3308,36 +3515,36 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="40" spans="1:60">
+    <row r="40" spans="1:72">
       <c r="A40">
         <v>45</v>
       </c>
       <c r="B40" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
       <c r="C40" t="s">
-        <v>278</v>
+        <v>290</v>
       </c>
       <c r="D40" t="s">
-        <v>279</v>
+        <v>291</v>
       </c>
       <c r="E40" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
       <c r="F40" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
       <c r="I40" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="J40">
         <v>400</v>
       </c>
       <c r="T40" t="s">
-        <v>281</v>
+        <v>293</v>
       </c>
       <c r="U40" t="s">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="AI40">
         <v>2000000</v>
@@ -3355,24 +3562,24 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="41" spans="1:60">
+    <row r="41" spans="1:72">
       <c r="A41">
         <v>46</v>
       </c>
       <c r="B41" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="C41" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
       <c r="D41" t="s">
-        <v>285</v>
+        <v>297</v>
       </c>
       <c r="E41" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="F41" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="AI41">
         <v>2500000</v>
@@ -3390,27 +3597,27 @@
         <v>8000</v>
       </c>
       <c r="BA41" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="42" spans="1:60">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="42" spans="1:72">
       <c r="A42">
         <v>47</v>
       </c>
       <c r="B42" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="C42" t="s">
-        <v>289</v>
+        <v>301</v>
       </c>
       <c r="D42" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="E42" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="F42" t="s">
-        <v>292</v>
+        <v>304</v>
       </c>
       <c r="AQ42">
         <v>100</v>
@@ -3431,27 +3638,27 @@
         <v>7</v>
       </c>
       <c r="BA42" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="43" spans="1:60">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="43" spans="1:72">
       <c r="A43">
         <v>48</v>
       </c>
       <c r="B43" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="C43" t="s">
-        <v>295</v>
+        <v>307</v>
       </c>
       <c r="D43" t="s">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="E43" t="s">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="F43" t="s">
-        <v>298</v>
+        <v>310</v>
       </c>
       <c r="AQ43">
         <v>100</v>
@@ -3466,39 +3673,39 @@
         <v>100</v>
       </c>
       <c r="AU43" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="AY43">
         <v>7</v>
       </c>
       <c r="BA43" t="s">
-        <v>293</v>
+        <v>305</v>
       </c>
       <c r="BB43">
         <v>1000</v>
       </c>
     </row>
-    <row r="44" spans="1:60">
+    <row r="44" spans="1:72">
       <c r="A44">
         <v>49</v>
       </c>
       <c r="B44" t="s">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="C44" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="D44" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="E44" t="s">
-        <v>302</v>
+        <v>314</v>
       </c>
       <c r="F44" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="T44" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="AQ44">
         <v>100</v>
@@ -3513,36 +3720,36 @@
         <v>100</v>
       </c>
       <c r="AU44" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="AY44">
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:60">
+    <row r="45" spans="1:72">
       <c r="A45">
         <v>50</v>
       </c>
       <c r="B45" t="s">
-        <v>305</v>
+        <v>317</v>
       </c>
       <c r="C45" t="s">
-        <v>306</v>
+        <v>318</v>
       </c>
       <c r="D45" t="s">
-        <v>307</v>
+        <v>319</v>
       </c>
       <c r="E45" t="s">
-        <v>308</v>
+        <v>320</v>
       </c>
       <c r="F45" t="s">
-        <v>308</v>
+        <v>320</v>
       </c>
       <c r="T45" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="U45" t="s">
-        <v>309</v>
+        <v>321</v>
       </c>
       <c r="AQ45">
         <v>100</v>
@@ -3557,33 +3764,33 @@
         <v>100</v>
       </c>
       <c r="AU45" t="s">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="AY45">
         <v>7</v>
       </c>
       <c r="BA45" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="46" spans="1:60">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="46" spans="1:72">
       <c r="A46">
         <v>51</v>
       </c>
       <c r="B46" t="s">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="C46" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="D46" t="s">
-        <v>312</v>
+        <v>324</v>
       </c>
       <c r="E46" t="s">
-        <v>313</v>
+        <v>325</v>
       </c>
       <c r="F46" t="s">
-        <v>314</v>
+        <v>326</v>
       </c>
       <c r="H46">
         <v>10</v>
@@ -3601,33 +3808,33 @@
         <v>2500</v>
       </c>
       <c r="AU46" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="47" spans="1:60">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="47" spans="1:72">
       <c r="A47">
         <v>52</v>
       </c>
       <c r="B47" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="C47" t="s">
-        <v>316</v>
+        <v>328</v>
       </c>
       <c r="D47" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
       <c r="E47" t="s">
-        <v>318</v>
+        <v>330</v>
       </c>
       <c r="F47" t="s">
-        <v>318</v>
+        <v>330</v>
       </c>
       <c r="S47" t="s">
-        <v>287</v>
+        <v>299</v>
       </c>
       <c r="T47" t="s">
-        <v>319</v>
+        <v>331</v>
       </c>
       <c r="AQ47">
         <v>100000</v>
@@ -3642,33 +3849,33 @@
         <v>10000</v>
       </c>
       <c r="AU47" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="48" spans="1:60">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="48" spans="1:72">
       <c r="A48">
         <v>53</v>
       </c>
       <c r="B48" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="C48" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
       <c r="D48" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
       <c r="E48" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
       <c r="F48" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
       <c r="T48" t="s">
-        <v>324</v>
+        <v>336</v>
       </c>
       <c r="U48" t="s">
-        <v>325</v>
+        <v>337</v>
       </c>
       <c r="AQ48">
         <v>10000</v>
@@ -3683,27 +3890,27 @@
         <v>10000</v>
       </c>
       <c r="AU48" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="49" spans="1:60">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="49" spans="1:72">
       <c r="A49">
         <v>54</v>
       </c>
       <c r="B49" t="s">
-        <v>326</v>
+        <v>338</v>
       </c>
       <c r="C49" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="D49" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="E49" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="F49" t="s">
-        <v>330</v>
+        <v>342</v>
       </c>
       <c r="AQ49">
         <v>100000</v>
@@ -3718,33 +3925,33 @@
         <v>25000</v>
       </c>
       <c r="AU49" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="BG49">
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:60">
+    <row r="50" spans="1:72">
       <c r="A50">
         <v>55</v>
       </c>
       <c r="B50" t="s">
-        <v>331</v>
+        <v>343</v>
       </c>
       <c r="C50" t="s">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="D50" t="s">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="E50" t="s">
-        <v>334</v>
+        <v>346</v>
       </c>
       <c r="F50" t="s">
-        <v>334</v>
+        <v>346</v>
       </c>
       <c r="U50" t="s">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="AQ50">
         <v>200000</v>
@@ -3759,7 +3966,7 @@
         <v>30000</v>
       </c>
       <c r="AU50" t="s">
-        <v>326</v>
+        <v>338</v>
       </c>
       <c r="BG50">
         <v>1</v>
@@ -3768,24 +3975,24 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:60">
+    <row r="51" spans="1:72">
       <c r="A51">
         <v>56</v>
       </c>
       <c r="B51" t="s">
-        <v>336</v>
+        <v>348</v>
       </c>
       <c r="C51" t="s">
-        <v>337</v>
+        <v>349</v>
       </c>
       <c r="D51" t="s">
-        <v>338</v>
+        <v>350</v>
       </c>
       <c r="E51" t="s">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="F51" t="s">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="AQ51">
         <v>500000</v>
@@ -3800,13 +4007,336 @@
         <v>125000</v>
       </c>
       <c r="AU51" t="s">
-        <v>331</v>
+        <v>343</v>
       </c>
       <c r="BG51">
         <v>2</v>
       </c>
       <c r="BH51">
         <v>10</v>
+      </c>
+    </row>
+    <row r="52" spans="1:72">
+      <c r="A52">
+        <v>57</v>
+      </c>
+      <c r="B52" t="s">
+        <v>352</v>
+      </c>
+      <c r="C52" t="s">
+        <v>353</v>
+      </c>
+      <c r="D52" t="s">
+        <v>354</v>
+      </c>
+      <c r="E52" t="s">
+        <v>355</v>
+      </c>
+      <c r="F52" t="s">
+        <v>356</v>
+      </c>
+      <c r="AQ52">
+        <v>2500</v>
+      </c>
+      <c r="AR52">
+        <v>1000</v>
+      </c>
+      <c r="AS52">
+        <v>2500</v>
+      </c>
+      <c r="AT52">
+        <v>150</v>
+      </c>
+      <c r="AU52" t="s">
+        <v>87</v>
+      </c>
+      <c r="BI52" t="s">
+        <v>357</v>
+      </c>
+      <c r="BJ52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:72">
+      <c r="A53">
+        <v>58</v>
+      </c>
+      <c r="B53" t="s">
+        <v>358</v>
+      </c>
+      <c r="C53" t="s">
+        <v>359</v>
+      </c>
+      <c r="D53" t="s">
+        <v>360</v>
+      </c>
+      <c r="E53" t="s">
+        <v>361</v>
+      </c>
+      <c r="F53" t="s">
+        <v>361</v>
+      </c>
+      <c r="AQ53">
+        <v>5000</v>
+      </c>
+      <c r="AR53">
+        <v>5000</v>
+      </c>
+      <c r="AS53">
+        <v>25000</v>
+      </c>
+      <c r="AT53">
+        <v>200</v>
+      </c>
+      <c r="AU53" t="s">
+        <v>96</v>
+      </c>
+      <c r="BI53" t="s">
+        <v>362</v>
+      </c>
+      <c r="BJ53">
+        <v>1</v>
+      </c>
+      <c r="BK53" t="s">
+        <v>363</v>
+      </c>
+      <c r="BL53" t="s">
+        <v>364</v>
+      </c>
+      <c r="BM53" t="s">
+        <v>365</v>
+      </c>
+      <c r="BN53">
+        <v>15</v>
+      </c>
+      <c r="BO53">
+        <v>1</v>
+      </c>
+      <c r="BP53" t="s">
+        <v>363</v>
+      </c>
+      <c r="BQ53" t="s">
+        <v>366</v>
+      </c>
+      <c r="BR53" t="s">
+        <v>367</v>
+      </c>
+      <c r="BS53">
+        <v>20</v>
+      </c>
+      <c r="BT53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:72">
+      <c r="A54">
+        <v>59</v>
+      </c>
+      <c r="B54" t="s">
+        <v>368</v>
+      </c>
+      <c r="C54" t="s">
+        <v>369</v>
+      </c>
+      <c r="D54" t="s">
+        <v>370</v>
+      </c>
+      <c r="E54" t="s">
+        <v>371</v>
+      </c>
+      <c r="F54" t="s">
+        <v>371</v>
+      </c>
+      <c r="AQ54">
+        <v>5000</v>
+      </c>
+      <c r="AR54">
+        <v>5000</v>
+      </c>
+      <c r="AS54">
+        <v>20000</v>
+      </c>
+      <c r="AT54">
+        <v>500</v>
+      </c>
+      <c r="AU54" t="s">
+        <v>187</v>
+      </c>
+      <c r="BI54" t="s">
+        <v>372</v>
+      </c>
+      <c r="BJ54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:72">
+      <c r="A55">
+        <v>60</v>
+      </c>
+      <c r="B55" t="s">
+        <v>373</v>
+      </c>
+      <c r="C55" t="s">
+        <v>374</v>
+      </c>
+      <c r="D55" t="s">
+        <v>375</v>
+      </c>
+      <c r="E55" t="s">
+        <v>376</v>
+      </c>
+      <c r="F55" t="s">
+        <v>376</v>
+      </c>
+      <c r="AQ55">
+        <v>2000</v>
+      </c>
+      <c r="AR55">
+        <v>1000</v>
+      </c>
+      <c r="AS55">
+        <v>175</v>
+      </c>
+      <c r="AT55">
+        <v>175</v>
+      </c>
+      <c r="AU55" t="s">
+        <v>103</v>
+      </c>
+      <c r="BI55" t="s">
+        <v>362</v>
+      </c>
+      <c r="BJ55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:72">
+      <c r="A56">
+        <v>61</v>
+      </c>
+      <c r="B56" t="s">
+        <v>377</v>
+      </c>
+      <c r="C56" t="s">
+        <v>378</v>
+      </c>
+      <c r="D56" t="s">
+        <v>379</v>
+      </c>
+      <c r="E56" t="s">
+        <v>380</v>
+      </c>
+      <c r="F56" t="s">
+        <v>380</v>
+      </c>
+      <c r="AQ56">
+        <v>5000</v>
+      </c>
+      <c r="AR56">
+        <v>5000</v>
+      </c>
+      <c r="AS56">
+        <v>10000</v>
+      </c>
+      <c r="AT56">
+        <v>1000</v>
+      </c>
+      <c r="AU56" t="s">
+        <v>368</v>
+      </c>
+      <c r="BK56" t="s">
+        <v>381</v>
+      </c>
+      <c r="BL56" t="s">
+        <v>382</v>
+      </c>
+      <c r="BM56" t="s">
+        <v>383</v>
+      </c>
+      <c r="BN56">
+        <v>25</v>
+      </c>
+      <c r="BO56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:72">
+      <c r="A57">
+        <v>62</v>
+      </c>
+      <c r="B57" t="s">
+        <v>384</v>
+      </c>
+      <c r="C57" t="s">
+        <v>385</v>
+      </c>
+      <c r="D57" t="s">
+        <v>386</v>
+      </c>
+      <c r="E57" t="s">
+        <v>387</v>
+      </c>
+      <c r="F57" t="s">
+        <v>387</v>
+      </c>
+      <c r="AQ57">
+        <v>5000</v>
+      </c>
+      <c r="AR57">
+        <v>5000</v>
+      </c>
+      <c r="AS57">
+        <v>2000</v>
+      </c>
+      <c r="AT57">
+        <v>350</v>
+      </c>
+      <c r="AU57" t="s">
+        <v>251</v>
+      </c>
+      <c r="BC57">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="58" spans="1:72">
+      <c r="A58">
+        <v>63</v>
+      </c>
+      <c r="B58" t="s">
+        <v>388</v>
+      </c>
+      <c r="C58" t="s">
+        <v>389</v>
+      </c>
+      <c r="D58" t="s">
+        <v>390</v>
+      </c>
+      <c r="E58" t="s">
+        <v>391</v>
+      </c>
+      <c r="F58" t="s">
+        <v>391</v>
+      </c>
+      <c r="AQ58">
+        <v>10000</v>
+      </c>
+      <c r="AR58">
+        <v>10000</v>
+      </c>
+      <c r="AS58">
+        <v>80000</v>
+      </c>
+      <c r="AT58">
+        <v>1000</v>
+      </c>
+      <c r="AU58" t="s">
+        <v>176</v>
+      </c>
+      <c r="BI58" t="s">
+        <v>392</v>
+      </c>
+      <c r="BJ58">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
The final steps are in place, now its cleanup and bug fix time
</commit_message>
<xml_diff>
--- a/resources/data-imports/Quests/guide-quests.xlsx
+++ b/resources/data-imports/Quests/guide-quests.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="395">
   <si>
     <t>id</t>
   </si>
@@ -168,6 +168,12 @@
   </si>
   <si>
     <t>required_event_goal_participation</t>
+  </si>
+  <si>
+    <t>required_event_goal_crafting_participation</t>
+  </si>
+  <si>
+    <t>required_event_goal_enchanting_participation</t>
   </si>
   <si>
     <t>required_holy_stacks</t>
@@ -1533,7 +1539,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:BT58"/>
+  <dimension ref="A1:BS58"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="3.428" bestFit="true" customWidth="true" style="0"/>
@@ -1583,34 +1589,33 @@
     <col min="45" max="45" width="13.997" bestFit="true" customWidth="true" style="0"/>
     <col min="46" max="46" width="11.711" bestFit="true" customWidth="true" style="0"/>
     <col min="47" max="47" width="43.561" bestFit="true" customWidth="true" style="0"/>
-    <col min="48" max="48" width="9.10" bestFit="true" style="0"/>
-    <col min="49" max="49" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="50" max="50" width="9.10" bestFit="true" style="0"/>
-    <col min="51" max="51" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="52" max="52" width="9.10" bestFit="true" style="0"/>
-    <col min="53" max="53" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="54" max="54" width="39.99" bestFit="true" customWidth="true" style="0"/>
-    <col min="55" max="55" width="24.708" bestFit="true" customWidth="true" style="0"/>
-    <col min="56" max="56" width="26.993" bestFit="true" customWidth="true" style="0"/>
-    <col min="57" max="57" width="28.136" bestFit="true" customWidth="true" style="0"/>
-    <col min="58" max="58" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="59" max="59" width="34.135" bestFit="true" customWidth="true" style="0"/>
-    <col min="60" max="60" width="29.421" bestFit="true" customWidth="true" style="0"/>
-    <col min="61" max="61" width="34.135" bestFit="true" customWidth="true" style="0"/>
-    <col min="62" max="62" width="35.277" bestFit="true" customWidth="true" style="0"/>
-    <col min="63" max="63" width="26.993" bestFit="true" customWidth="true" style="0"/>
-    <col min="64" max="64" width="29.421" bestFit="true" customWidth="true" style="0"/>
-    <col min="65" max="65" width="28.136" bestFit="true" customWidth="true" style="0"/>
-    <col min="66" max="66" width="26.993" bestFit="true" customWidth="true" style="0"/>
-    <col min="67" max="67" width="39.99" bestFit="true" customWidth="true" style="0"/>
-    <col min="68" max="68" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="48" max="48" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="49" max="49" width="21.138" bestFit="true" customWidth="true" style="0"/>
+    <col min="50" max="50" width="23.423" bestFit="true" customWidth="true" style="0"/>
+    <col min="51" max="51" width="39.99" bestFit="true" customWidth="true" style="0"/>
+    <col min="52" max="52" width="50.559" bestFit="true" customWidth="true" style="0"/>
+    <col min="53" max="53" width="52.987" bestFit="true" customWidth="true" style="0"/>
+    <col min="54" max="54" width="24.708" bestFit="true" customWidth="true" style="0"/>
+    <col min="55" max="55" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="56" max="56" width="28.136" bestFit="true" customWidth="true" style="0"/>
+    <col min="57" max="57" width="23.423" bestFit="true" customWidth="true" style="0"/>
+    <col min="58" max="58" width="34.135" bestFit="true" customWidth="true" style="0"/>
+    <col min="59" max="59" width="29.421" bestFit="true" customWidth="true" style="0"/>
+    <col min="60" max="60" width="34.135" bestFit="true" customWidth="true" style="0"/>
+    <col min="61" max="61" width="35.277" bestFit="true" customWidth="true" style="0"/>
+    <col min="62" max="62" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="63" max="63" width="29.421" bestFit="true" customWidth="true" style="0"/>
+    <col min="64" max="64" width="28.136" bestFit="true" customWidth="true" style="0"/>
+    <col min="65" max="65" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="66" max="66" width="39.99" bestFit="true" customWidth="true" style="0"/>
+    <col min="67" max="67" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="68" max="68" width="24.708" bestFit="true" customWidth="true" style="0"/>
     <col min="69" max="69" width="24.708" bestFit="true" customWidth="true" style="0"/>
-    <col min="70" max="70" width="24.708" bestFit="true" customWidth="true" style="0"/>
-    <col min="71" max="71" width="26.993" bestFit="true" customWidth="true" style="0"/>
-    <col min="72" max="72" width="39.99" bestFit="true" customWidth="true" style="0"/>
+    <col min="70" max="70" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="71" max="71" width="39.99" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:72">
+    <row r="1" spans="1:71">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1752,91 +1757,97 @@
       <c r="AU1" t="s">
         <v>46</v>
       </c>
+      <c r="AV1" t="s">
+        <v>47</v>
+      </c>
       <c r="AW1" t="s">
-        <v>47</v>
+        <v>48</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>49</v>
       </c>
       <c r="AY1" t="s">
-        <v>48</v>
+        <v>50</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>51</v>
       </c>
       <c r="BA1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="BB1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="BC1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="BD1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="BE1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="BF1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="BG1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="BH1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="BI1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="BJ1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="BK1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="BL1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="BM1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="BN1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="BO1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="BP1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="BQ1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="BR1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="BS1" t="s">
-        <v>67</v>
-      </c>
-      <c r="BT1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="2" spans="1:72">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:71">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G2">
         <v>2</v>
@@ -1848,30 +1859,30 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:72">
+    <row r="3" spans="1:71">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G3">
         <v>10</v>
       </c>
       <c r="Q3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="R3">
         <v>1</v>
@@ -1883,36 +1894,36 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:72">
+    <row r="4" spans="1:71">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G4">
         <v>30</v>
       </c>
       <c r="I4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="J4">
         <v>10</v>
       </c>
       <c r="K4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="L4">
         <v>15</v>
@@ -1927,45 +1938,45 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:72">
+    <row r="5" spans="1:71">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G5">
         <v>50</v>
       </c>
       <c r="I5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="J5">
         <v>5</v>
       </c>
       <c r="K5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="U5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="V5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AS5">
         <v>1000</v>
@@ -1974,42 +1985,42 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:72">
+    <row r="6" spans="1:71">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G6">
         <v>60</v>
       </c>
       <c r="I6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="J6">
         <v>5</v>
       </c>
       <c r="K6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="L6">
         <v>15</v>
       </c>
       <c r="U6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="AM6">
         <v>125</v>
@@ -2021,36 +2032,36 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:72">
+    <row r="7" spans="1:71">
       <c r="A7">
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G7">
         <v>120</v>
       </c>
       <c r="I7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="J7">
         <v>15</v>
       </c>
       <c r="K7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L7">
         <v>5</v>
@@ -2062,7 +2073,7 @@
         <v>10</v>
       </c>
       <c r="U7" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="X7">
         <v>500</v>
@@ -2083,33 +2094,33 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:72">
+    <row r="8" spans="1:71">
       <c r="A8">
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E8" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F8" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="Q8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="R8">
         <v>3</v>
       </c>
       <c r="T8" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AQ8">
         <v>1000</v>
@@ -2124,33 +2135,33 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:72">
+    <row r="9" spans="1:71">
       <c r="A9">
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C9" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D9" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I9" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="J9">
         <v>50</v>
       </c>
       <c r="T9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="AQ9">
         <v>2500</v>
@@ -2165,39 +2176,39 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:72">
+    <row r="10" spans="1:71">
       <c r="A10">
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C10" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D10" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E10" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F10" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G10">
         <v>300</v>
       </c>
       <c r="Q10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="R10">
         <v>2</v>
       </c>
       <c r="S10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="U10" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="AQ10">
         <v>1000</v>
@@ -2209,24 +2220,24 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:72">
+    <row r="11" spans="1:71">
       <c r="A11">
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C11" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E11" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="O11">
         <v>1</v>
@@ -2241,24 +2252,24 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="1:72">
+    <row r="12" spans="1:71">
       <c r="A12">
         <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C12" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E12" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F12" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="AB12">
         <v>1</v>
@@ -2276,33 +2287,33 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:72">
+    <row r="13" spans="1:71">
       <c r="A13">
         <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C13" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D13" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E13" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F13" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="I13" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="J13">
         <v>25</v>
       </c>
       <c r="K13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="L13">
         <v>5</v>
@@ -2314,7 +2325,7 @@
         <v>500</v>
       </c>
       <c r="AG13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="AH13">
         <v>1</v>
@@ -2326,24 +2337,24 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:72">
+    <row r="14" spans="1:71">
       <c r="A14">
         <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C14" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D14" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E14" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F14" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="AC14">
         <v>75</v>
@@ -2352,7 +2363,7 @@
         <v>2000</v>
       </c>
       <c r="AG14" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AH14">
         <v>2</v>
@@ -2364,33 +2375,33 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:72">
+    <row r="15" spans="1:71">
       <c r="A15">
         <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C15" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D15" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E15" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F15" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="I15" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="J15">
         <v>25</v>
       </c>
       <c r="K15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L15">
         <v>50</v>
@@ -2402,7 +2413,7 @@
         <v>10</v>
       </c>
       <c r="T15" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="AC15">
         <v>100</v>
@@ -2411,7 +2422,7 @@
         <v>3000</v>
       </c>
       <c r="AG15" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="AH15">
         <v>1</v>
@@ -2423,36 +2434,36 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="1:72">
+    <row r="16" spans="1:71">
       <c r="A16">
         <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C16" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D16" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E16" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F16" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G16">
         <v>500</v>
       </c>
       <c r="I16" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="J16">
         <v>100</v>
       </c>
       <c r="K16" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L16">
         <v>50</v>
@@ -2464,22 +2475,22 @@
         <v>100</v>
       </c>
       <c r="Q16" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="R16">
         <v>3</v>
       </c>
       <c r="S16" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="T16" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="U16" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="V16" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="X16">
         <v>25000</v>
@@ -2494,30 +2505,30 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" spans="1:72">
+    <row r="17" spans="1:71">
       <c r="A17">
         <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C17" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D17" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="E17" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F17" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="G17">
         <v>600</v>
       </c>
       <c r="I17" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="J17">
         <v>3</v>
@@ -2541,30 +2552,30 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:72">
+    <row r="18" spans="1:71">
       <c r="A18">
         <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C18" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D18" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E18" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F18" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G18">
         <v>1000</v>
       </c>
       <c r="K18" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L18">
         <v>400</v>
@@ -2582,7 +2593,7 @@
         <v>30</v>
       </c>
       <c r="T18" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="AI18">
         <v>6000</v>
@@ -2600,39 +2611,39 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="19" spans="1:72">
+    <row r="19" spans="1:71">
       <c r="A19">
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C19" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D19" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E19" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F19" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G19">
         <v>1500</v>
       </c>
       <c r="Q19" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="R19">
         <v>2</v>
       </c>
       <c r="S19" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="U19" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="AI19">
         <v>7000</v>
@@ -2644,30 +2655,30 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="20" spans="1:72">
+    <row r="20" spans="1:71">
       <c r="A20">
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C20" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D20" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E20" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F20" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="G20">
         <v>2000</v>
       </c>
       <c r="T20" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="AS20">
         <v>2000000000</v>
@@ -2676,30 +2687,30 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="21" spans="1:72">
+    <row r="21" spans="1:71">
       <c r="A21">
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C21" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D21" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E21" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F21" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G21">
         <v>2500</v>
       </c>
       <c r="I21" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="J21">
         <v>50</v>
@@ -2711,7 +2722,7 @@
         <v>50</v>
       </c>
       <c r="Q21" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="R21">
         <v>5</v>
@@ -2726,7 +2737,7 @@
         <v>20000</v>
       </c>
       <c r="AE21" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="AF21">
         <v>5</v>
@@ -2744,24 +2755,24 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="22" spans="1:72">
+    <row r="22" spans="1:71">
       <c r="A22">
         <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C22" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D22" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E22" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F22" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="AS22">
         <v>100000</v>
@@ -2769,34 +2780,34 @@
       <c r="AT22">
         <v>50</v>
       </c>
+      <c r="AV22">
+        <v>25</v>
+      </c>
       <c r="AW22">
-        <v>25</v>
-      </c>
-      <c r="AY22">
         <v>3</v>
       </c>
-      <c r="BA22" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="23" spans="1:72">
+      <c r="AX22" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="23" spans="1:71">
       <c r="A23">
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C23" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D23" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E23" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="F23" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="AS23">
         <v>100000</v>
@@ -2805,39 +2816,39 @@
         <v>75</v>
       </c>
       <c r="AU23" t="s">
-        <v>191</v>
+        <v>193</v>
+      </c>
+      <c r="AV23">
+        <v>25</v>
       </c>
       <c r="AW23">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="AY23">
-        <v>3</v>
-      </c>
-      <c r="BB23">
         <v>1000</v>
       </c>
     </row>
-    <row r="24" spans="1:72">
+    <row r="24" spans="1:71">
       <c r="A24">
         <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C24" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D24" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E24" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F24" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="T24" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="AQ24">
         <v>5000</v>
@@ -2852,36 +2863,36 @@
         <v>100</v>
       </c>
       <c r="AU24" t="s">
-        <v>191</v>
+        <v>193</v>
+      </c>
+      <c r="AV24">
+        <v>25</v>
       </c>
       <c r="AW24">
-        <v>25</v>
-      </c>
-      <c r="AY24">
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:72">
+    <row r="25" spans="1:71">
       <c r="A25">
         <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C25" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D25" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E25" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F25" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="T25" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="AQ25">
         <v>1000</v>
@@ -2896,36 +2907,36 @@
         <v>100</v>
       </c>
       <c r="AU25" t="s">
-        <v>202</v>
+        <v>204</v>
+      </c>
+      <c r="AV25">
+        <v>25</v>
       </c>
       <c r="AW25">
-        <v>25</v>
-      </c>
-      <c r="AY25">
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:72">
+    <row r="26" spans="1:71">
       <c r="A26">
         <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C26" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D26" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E26" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F26" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="T26" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="AQ26">
         <v>2000</v>
@@ -2940,36 +2951,36 @@
         <v>100</v>
       </c>
       <c r="AU26" t="s">
-        <v>191</v>
+        <v>193</v>
+      </c>
+      <c r="AV26">
+        <v>25</v>
       </c>
       <c r="AW26">
-        <v>25</v>
-      </c>
-      <c r="AY26">
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:72">
+    <row r="27" spans="1:71">
       <c r="A27">
         <v>32</v>
       </c>
       <c r="B27" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C27" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D27" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E27" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="F27" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="T27" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="AB27">
         <v>1</v>
@@ -2981,7 +2992,7 @@
         <v>500</v>
       </c>
       <c r="AG27" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="AH27">
         <v>1</v>
@@ -2999,42 +3010,42 @@
         <v>100</v>
       </c>
       <c r="AU27" t="s">
-        <v>191</v>
+        <v>193</v>
+      </c>
+      <c r="AV27">
+        <v>25</v>
       </c>
       <c r="AW27">
-        <v>25</v>
-      </c>
-      <c r="AY27">
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:72">
+    <row r="28" spans="1:71">
       <c r="A28">
         <v>33</v>
       </c>
       <c r="B28" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C28" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D28" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E28" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F28" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="S28" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="T28" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="U28" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="AQ28">
         <v>25000</v>
@@ -3048,31 +3059,31 @@
       <c r="AT28">
         <v>2000</v>
       </c>
-      <c r="BA28" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="29" spans="1:72">
+      <c r="AX28" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="29" spans="1:71">
       <c r="A29">
         <v>34</v>
       </c>
       <c r="B29" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C29" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D29" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E29" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="F29" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="Q29" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="R29">
         <v>2</v>
@@ -3089,31 +3100,31 @@
       <c r="AT29">
         <v>2000</v>
       </c>
-      <c r="BE29" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="30" spans="1:72">
+      <c r="BD29" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="30" spans="1:71">
       <c r="A30">
         <v>35</v>
       </c>
       <c r="B30" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C30" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D30" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E30" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F30" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="Q30" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="R30">
         <v>5</v>
@@ -3131,30 +3142,30 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="31" spans="1:72">
+    <row r="31" spans="1:71">
       <c r="A31">
         <v>36</v>
       </c>
       <c r="B31" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C31" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D31" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E31" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="F31" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="S31" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="T31" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="AQ31">
         <v>25000</v>
@@ -3168,31 +3179,31 @@
       <c r="AT31">
         <v>2000</v>
       </c>
-      <c r="BA31" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="32" spans="1:72">
+      <c r="AX31" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="32" spans="1:71">
       <c r="A32">
         <v>37</v>
       </c>
       <c r="B32" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C32" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D32" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E32" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F32" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="I32" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="J32">
         <v>200</v>
@@ -3210,27 +3221,27 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="33" spans="1:72">
+    <row r="33" spans="1:71">
       <c r="A33">
         <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C33" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="D33" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E33" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F33" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="T33" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="Z33">
         <v>5000</v>
@@ -3247,28 +3258,28 @@
       <c r="AT33">
         <v>5000</v>
       </c>
-      <c r="BC33">
+      <c r="BB33">
         <v>40</v>
       </c>
     </row>
-    <row r="34" spans="1:72">
+    <row r="34" spans="1:71">
       <c r="A34">
         <v>39</v>
       </c>
       <c r="B34" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C34" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D34" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E34" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="F34" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="AQ34">
         <v>50000</v>
@@ -3282,31 +3293,31 @@
       <c r="AT34">
         <v>5000</v>
       </c>
-      <c r="BE34" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="35" spans="1:72">
+      <c r="BD34" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="35" spans="1:71">
       <c r="A35">
         <v>40</v>
       </c>
       <c r="B35" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C35" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D35" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E35" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="F35" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="I35" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="J35">
         <v>25</v>
@@ -3324,27 +3335,27 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="36" spans="1:72">
+    <row r="36" spans="1:71">
       <c r="A36">
         <v>41</v>
       </c>
       <c r="B36" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C36" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D36" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E36" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="F36" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="Q36" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="R36">
         <v>5</v>
@@ -3361,40 +3372,40 @@
       <c r="AT36">
         <v>100</v>
       </c>
-      <c r="AW36">
+      <c r="AV36">
         <v>1500</v>
       </c>
-      <c r="BF36">
+      <c r="BE36">
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:72">
+    <row r="37" spans="1:71">
       <c r="A37">
         <v>42</v>
       </c>
       <c r="B37" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C37" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D37" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E37" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="F37" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="I37" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="J37">
         <v>75</v>
       </c>
       <c r="T37" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="AQ37">
         <v>150000</v>
@@ -3409,27 +3420,27 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="38" spans="1:72">
+    <row r="38" spans="1:71">
       <c r="A38">
         <v>43</v>
       </c>
       <c r="B38" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C38" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="D38" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E38" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="F38" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I38" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="J38">
         <v>150</v>
@@ -3450,13 +3461,13 @@
         <v>50000</v>
       </c>
       <c r="AE38" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="AF38">
         <v>30</v>
       </c>
       <c r="AG38" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="AH38">
         <v>4</v>
@@ -3474,27 +3485,27 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="39" spans="1:72">
+    <row r="39" spans="1:71">
       <c r="A39">
         <v>44</v>
       </c>
       <c r="B39" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C39" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="D39" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="E39" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="F39" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="I39" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="J39">
         <v>300</v>
@@ -3515,36 +3526,36 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="40" spans="1:72">
+    <row r="40" spans="1:71">
       <c r="A40">
         <v>45</v>
       </c>
       <c r="B40" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C40" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D40" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E40" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="F40" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="I40" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="J40">
         <v>400</v>
       </c>
       <c r="T40" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="U40" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="AI40">
         <v>2000000</v>
@@ -3562,24 +3573,24 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="41" spans="1:72">
+    <row r="41" spans="1:71">
       <c r="A41">
         <v>46</v>
       </c>
       <c r="B41" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C41" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D41" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E41" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="F41" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AI41">
         <v>2500000</v>
@@ -3596,28 +3607,28 @@
       <c r="AT41">
         <v>8000</v>
       </c>
-      <c r="BA41" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="42" spans="1:72">
+      <c r="AX41" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="42" spans="1:71">
       <c r="A42">
         <v>47</v>
       </c>
       <c r="B42" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C42" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="D42" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E42" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="F42" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="AQ42">
         <v>100</v>
@@ -3631,34 +3642,34 @@
       <c r="AT42">
         <v>100</v>
       </c>
+      <c r="AV42">
+        <v>10</v>
+      </c>
       <c r="AW42">
-        <v>10</v>
-      </c>
-      <c r="AY42">
         <v>7</v>
       </c>
-      <c r="BA42" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="43" spans="1:72">
+      <c r="AX42" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="43" spans="1:71">
       <c r="A43">
         <v>48</v>
       </c>
       <c r="B43" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="C43" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D43" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E43" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="F43" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="AQ43">
         <v>100</v>
@@ -3673,39 +3684,39 @@
         <v>100</v>
       </c>
       <c r="AU43" t="s">
-        <v>300</v>
+        <v>302</v>
+      </c>
+      <c r="AW43">
+        <v>7</v>
+      </c>
+      <c r="AX43" t="s">
+        <v>307</v>
       </c>
       <c r="AY43">
-        <v>7</v>
-      </c>
-      <c r="BA43" t="s">
-        <v>305</v>
-      </c>
-      <c r="BB43">
         <v>1000</v>
       </c>
     </row>
-    <row r="44" spans="1:72">
+    <row r="44" spans="1:71">
       <c r="A44">
         <v>49</v>
       </c>
       <c r="B44" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C44" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="D44" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E44" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="F44" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="T44" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="AQ44">
         <v>100</v>
@@ -3720,36 +3731,36 @@
         <v>100</v>
       </c>
       <c r="AU44" t="s">
-        <v>306</v>
-      </c>
-      <c r="AY44">
+        <v>308</v>
+      </c>
+      <c r="AW44">
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:72">
+    <row r="45" spans="1:71">
       <c r="A45">
         <v>50</v>
       </c>
       <c r="B45" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C45" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="D45" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="E45" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="F45" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="T45" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="U45" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="AQ45">
         <v>100</v>
@@ -3764,33 +3775,33 @@
         <v>100</v>
       </c>
       <c r="AU45" t="s">
-        <v>311</v>
-      </c>
-      <c r="AY45">
+        <v>313</v>
+      </c>
+      <c r="AW45">
         <v>7</v>
       </c>
-      <c r="BA45" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="46" spans="1:72">
+      <c r="AX45" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="46" spans="1:71">
       <c r="A46">
         <v>51</v>
       </c>
       <c r="B46" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C46" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="D46" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="E46" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="F46" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="H46">
         <v>10</v>
@@ -3808,33 +3819,33 @@
         <v>2500</v>
       </c>
       <c r="AU46" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="47" spans="1:72">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="47" spans="1:71">
       <c r="A47">
         <v>52</v>
       </c>
       <c r="B47" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C47" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D47" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E47" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="F47" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="S47" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="T47" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="AQ47">
         <v>100000</v>
@@ -3849,33 +3860,33 @@
         <v>10000</v>
       </c>
       <c r="AU47" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="48" spans="1:72">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="48" spans="1:71">
       <c r="A48">
         <v>53</v>
       </c>
       <c r="B48" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="C48" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="D48" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="E48" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="F48" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="T48" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="U48" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="AQ48">
         <v>10000</v>
@@ -3890,27 +3901,27 @@
         <v>10000</v>
       </c>
       <c r="AU48" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="49" spans="1:72">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="49" spans="1:71">
       <c r="A49">
         <v>54</v>
       </c>
       <c r="B49" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="C49" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="D49" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="E49" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="F49" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="AQ49">
         <v>100000</v>
@@ -3925,33 +3936,33 @@
         <v>25000</v>
       </c>
       <c r="AU49" t="s">
-        <v>332</v>
-      </c>
-      <c r="BG49">
+        <v>334</v>
+      </c>
+      <c r="BF49">
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:72">
+    <row r="50" spans="1:71">
       <c r="A50">
         <v>55</v>
       </c>
       <c r="B50" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C50" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D50" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="E50" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="F50" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="U50" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="AQ50">
         <v>200000</v>
@@ -3966,33 +3977,33 @@
         <v>30000</v>
       </c>
       <c r="AU50" t="s">
-        <v>338</v>
+        <v>340</v>
+      </c>
+      <c r="BF50">
+        <v>1</v>
       </c>
       <c r="BG50">
-        <v>1</v>
-      </c>
-      <c r="BH50">
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:72">
+    <row r="51" spans="1:71">
       <c r="A51">
         <v>56</v>
       </c>
       <c r="B51" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C51" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="D51" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="E51" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="F51" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="AQ51">
         <v>500000</v>
@@ -4007,33 +4018,33 @@
         <v>125000</v>
       </c>
       <c r="AU51" t="s">
-        <v>343</v>
+        <v>345</v>
+      </c>
+      <c r="BF51">
+        <v>2</v>
       </c>
       <c r="BG51">
-        <v>2</v>
-      </c>
-      <c r="BH51">
         <v>10</v>
       </c>
     </row>
-    <row r="52" spans="1:72">
+    <row r="52" spans="1:71">
       <c r="A52">
         <v>57</v>
       </c>
       <c r="B52" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="C52" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="D52" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="E52" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F52" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="AQ52">
         <v>2500</v>
@@ -4048,33 +4059,33 @@
         <v>150</v>
       </c>
       <c r="AU52" t="s">
-        <v>87</v>
-      </c>
-      <c r="BI52" t="s">
-        <v>357</v>
-      </c>
-      <c r="BJ52">
+        <v>89</v>
+      </c>
+      <c r="BH52" t="s">
+        <v>359</v>
+      </c>
+      <c r="BI52">
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:72">
+    <row r="53" spans="1:71">
       <c r="A53">
         <v>58</v>
       </c>
       <c r="B53" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C53" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="D53" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="E53" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="F53" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="AQ53">
         <v>5000</v>
@@ -4089,63 +4100,63 @@
         <v>200</v>
       </c>
       <c r="AU53" t="s">
-        <v>96</v>
-      </c>
-      <c r="BI53" t="s">
-        <v>362</v>
-      </c>
-      <c r="BJ53">
+        <v>98</v>
+      </c>
+      <c r="BH53" t="s">
+        <v>364</v>
+      </c>
+      <c r="BI53">
         <v>1</v>
       </c>
+      <c r="BJ53" t="s">
+        <v>365</v>
+      </c>
       <c r="BK53" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="BL53" t="s">
-        <v>364</v>
-      </c>
-      <c r="BM53" t="s">
+        <v>367</v>
+      </c>
+      <c r="BM53">
+        <v>15</v>
+      </c>
+      <c r="BN53">
+        <v>1</v>
+      </c>
+      <c r="BO53" t="s">
         <v>365</v>
       </c>
-      <c r="BN53">
-        <v>15</v>
-      </c>
-      <c r="BO53">
-        <v>1</v>
-      </c>
       <c r="BP53" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="BQ53" t="s">
-        <v>366</v>
-      </c>
-      <c r="BR53" t="s">
-        <v>367</v>
+        <v>369</v>
+      </c>
+      <c r="BR53">
+        <v>20</v>
       </c>
       <c r="BS53">
-        <v>20</v>
-      </c>
-      <c r="BT53">
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:72">
+    <row r="54" spans="1:71">
       <c r="A54">
         <v>59</v>
       </c>
       <c r="B54" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C54" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="D54" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="E54" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="F54" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="AQ54">
         <v>5000</v>
@@ -4160,33 +4171,33 @@
         <v>500</v>
       </c>
       <c r="AU54" t="s">
-        <v>187</v>
-      </c>
-      <c r="BI54" t="s">
-        <v>372</v>
-      </c>
-      <c r="BJ54">
+        <v>189</v>
+      </c>
+      <c r="BH54" t="s">
+        <v>374</v>
+      </c>
+      <c r="BI54">
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:72">
+    <row r="55" spans="1:71">
       <c r="A55">
         <v>60</v>
       </c>
       <c r="B55" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="C55" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="D55" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E55" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="F55" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="AQ55">
         <v>2000</v>
@@ -4201,33 +4212,33 @@
         <v>175</v>
       </c>
       <c r="AU55" t="s">
-        <v>103</v>
-      </c>
-      <c r="BI55" t="s">
-        <v>362</v>
-      </c>
-      <c r="BJ55">
+        <v>105</v>
+      </c>
+      <c r="BH55" t="s">
+        <v>364</v>
+      </c>
+      <c r="BI55">
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:72">
+    <row r="56" spans="1:71">
       <c r="A56">
         <v>61</v>
       </c>
       <c r="B56" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="C56" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="D56" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="E56" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="F56" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="AQ56">
         <v>5000</v>
@@ -4242,42 +4253,42 @@
         <v>1000</v>
       </c>
       <c r="AU56" t="s">
-        <v>368</v>
+        <v>370</v>
+      </c>
+      <c r="BJ56" t="s">
+        <v>383</v>
       </c>
       <c r="BK56" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="BL56" t="s">
-        <v>382</v>
-      </c>
-      <c r="BM56" t="s">
-        <v>383</v>
+        <v>385</v>
+      </c>
+      <c r="BM56">
+        <v>25</v>
       </c>
       <c r="BN56">
-        <v>25</v>
-      </c>
-      <c r="BO56">
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:72">
+    <row r="57" spans="1:71">
       <c r="A57">
         <v>62</v>
       </c>
       <c r="B57" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="C57" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="D57" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="E57" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="F57" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="AQ57">
         <v>5000</v>
@@ -4292,30 +4303,30 @@
         <v>350</v>
       </c>
       <c r="AU57" t="s">
-        <v>251</v>
-      </c>
-      <c r="BC57">
+        <v>253</v>
+      </c>
+      <c r="BB57">
         <v>80</v>
       </c>
     </row>
-    <row r="58" spans="1:72">
+    <row r="58" spans="1:71">
       <c r="A58">
         <v>63</v>
       </c>
       <c r="B58" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="C58" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="D58" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="E58" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="F58" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="AQ58">
         <v>10000</v>
@@ -4330,12 +4341,12 @@
         <v>1000</v>
       </c>
       <c r="AU58" t="s">
-        <v>176</v>
-      </c>
-      <c r="BI58" t="s">
-        <v>392</v>
-      </c>
-      <c r="BJ58">
+        <v>178</v>
+      </c>
+      <c r="BH58" t="s">
+        <v>394</v>
+      </c>
+      <c r="BI58">
         <v>1</v>
       </c>
     </row>

</xml_diff>